<commit_message>
second commit to xhs spider.
</commit_message>
<xml_diff>
--- a/南京 吃_小红书旅游笔记.xlsx
+++ b/南京 吃_小红书旅游笔记.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +425,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>标题</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>作者</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>图片链接</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>点赞数</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>链接</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>南京没有任何环境但每次来必吃的压箱底神店</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>南京没有任何环境但每次来必吃的压箱底神店
+每次来南京巡演真的必吃，建议去之前打电话询问一下
+#吃什么 #美食日常 #本地人带你吃 #南京 #南京美食 #南京探店 #南京旅游 #吃货薯 #吃货日常
+4小时前 江苏</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/search_result/684c09e6000000002001ed17?xsec_token=ABDvhwY4XJpE8GjP93PDei2CI3ui4i_70cPRkZdUpY8EY=&amp;xsec_source=</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>南京这家真的好好吃！！！（超大声😭😭</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>南京这家真的好好吃！！！（超大声😭😭
+藏在明瓦廊的神仙川菜馆！！！
+人均只要五六十，性价比高到飞起～
+分量还感人，我怎么才知道
+他家简直就是米饭杀手！！王牌鸡爪✔️泡椒土豆丝✔️敲下饭！还有新上的罗氏虾🦐爱上鲍鱼✔️简直是我的心头好，虾大肉厚，鲜美入味，每一口都hin满足！
+除了要排队👫👭👬
+真的挑不出一点毛病（图2️⃣是工作日晚上九点的排队状态）
+#我是国庆知食分子 #国庆逛吃日记 #小滋味城市大选 #我超爱的穷鬼小店#国庆划得来逛吃指南 #大声安利本地美食 #最强美食城市安利 #平价美食 #走街串巷找美食 #川菜 #大声安利本地美食   #发现一家南京好店  #南京旅游攻略  #川菜馆 #南京川菜   #南京新街口美食 #不怕辣最爱的川菜
+2024-09-27</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://sns-webpic-qc.xhscdn.com/202506132347/b4c8686370794876541bc606117e26b9/1040g0083187v2f6e0o005p4ee0fnor6knbn0g70!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/de46526446ef0c8c9b36b3697d8dbc9a/1040g0083187v2f6e0o305p4ee0fnor6k8eriec8!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/0c20f33d945cea47bf91d256100b3c44/1040g0083187v2f6e0o105p4ee0fnor6ksatul6g!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/989fc147684e82cdd946375bf911a9e6/1040g0083187v2f6e0o0g5p4ee0fnor6k5oi5mp0!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/55d5706ad67822445c3933c9bf9b5415/1040g0083187v2f6e0o1g5p4ee0fnor6kv71d0ko!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/f5892a6a80c422b197a80bd2a3146f16/1040g0083187v2f6e0o3g5p4ee0fnor6kqi1qf2g!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/696dc3640defa6e1261bc0b2a31a2349/1040g0083187v2f6e0o2g5p4ee0fnor6kehhqtro!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/f4deda37dfe5878c7d3a6ace76209436/1040g0083187v2f6e0o4g5p4ee0fnor6k9aog9vo!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/ed1b1a4521eb0571aea25f44c485bc79/1040g0083187v2f6e0o405p4ee0fnor6k8n9rr10!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/cc547be7afa13acc6967deea3b937037/1040g0083187v2f6e0o205p4ee0fnor6kksm92s8!nd_dft_wlteh_webp_3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/search_result/66f60af2000000001b021e6a?xsec_token=ABfquRLsximqipcQlhEavUjNgR9sM-ZWL6dUZPB92LeT4=&amp;xsec_source=</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>我在南京吃过最好吃的牛肉锅贴🥟‼️</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>我在南京吃过最好吃的牛肉锅贴🥟‼️
+⏰今天接小孩放学的时候正好下雨，就在学校附近找了一家餐馆，随便吃一点！
+🥢🍴 牛肉锅贴：外皮超酥脆，一口咬下去嘎嘣脆，肉质特别鲜嫩，真的会爆汁的那种～
+🍲🥩 除了牛肉锅贴，他们家的红烧牛肉炒和红烧牛肉汤面也是一绝。原汁原味的牛肉汤底，配上红烧牛肉做浇头，牛肉炖的又酥又烂，入口即化，这一大碗面比我的脸都大，真的是货真价实，实实在在～
+💖📣 这家店便宜又好吃，真的是一个很不错的选，附近的小伙伴们觉得我说得对吗？
+#王务民牛肉汤馆 #锅贴 #红烧牛肉面 #红烧牛肉汤面 #面条嗦面 #条条小马路都好吃 #这家店我从小吃到大 #南京美食灵感日记 #本地人才知道的美食 #牛肉面 @薯队长 @吃货薯
+2小时前 江苏</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://sns-webpic-qc.xhscdn.com/202506132347/12311b2684677460557c0594896c3a42/notes_pre_post/1040g3k031im20j091e5g5oflc7b40k2balq36d8!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/e863c8dad1eb20108d68cdb15c7f768f/notes_pre_post/1040g3k031im20j091e405oflc7b40k2b0u0fdg0!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/812418379630bd34b81d558e0d666909/notes_pre_post/1040g3k031im20j091e6g5oflc7b40k2bhfcgpjo!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/a89c2f6bba876800e4496f980ee87322/notes_pre_post/1040g3k031im20j091e4g5oflc7b40k2brf20ul8!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/e8f8337238c2090b2afc2e0db87fa651/notes_pre_post/1040g3k031im20j091e3g5oflc7b40k2b78ppdeg!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/3cd60f55039ce1d9fdd1d9e0128b777c/notes_pre_post/1040g3k031im20j091e605oflc7b40k2bkoughr0!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/d4ab48b80932ac7f90b4e82d142065cc/notes_pre_post/1040g3k831im29o8sh4205oflc7b40k2bmnktvk8!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/5b52278a129dbfd0941c3cbd20435784/notes_pre_post/1040g3k031im20j091e505oflc7b40k2b7d7sm8g!nd_dft_wlteh_webp_3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/search_result/684c2b4a000000002102f07a?xsec_token=ABDvhwY4XJpE8GjP93PDei2PweTrgbJFA24P_5AvCSS4g=&amp;xsec_source=</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>在南京半天怒吃五家店❗️太好吃了我服了！</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>在南京半天怒吃五家店❗️太好吃了我服了！
+之前就想出的！4家我吃了超多次宝藏小店！一家跟风乌啦啦的大肉面！都非常好吃！一天可以全部打卡完！南京真的太好吃了！下次还来！（第一次尝试拍合集，不足的地方大家见谅！欢迎大家给俺提建议！）﻿#南京美食﻿ ﻿#我家的春天真好吃﻿ ﻿#藏在小馆里的春和景明﻿ ﻿#南京探店﻿ ﻿#南京﻿ ﻿#敢敢的饭桶日记﻿ ﻿#烤鸭﻿ ﻿#汤包﻿ ﻿#大肉面
+03-06</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/search_result/67c945c80000000029032ccc?xsec_token=ABZJh4LXDd3KO76JSSnDyvzdaKpQx2t3VoYOkvTeM2yqM=&amp;xsec_source=</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>我真的很需要无广南京美食推荐啊啊啊啊啊啊</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>我真的很需要无广南京美食推荐啊啊啊啊啊啊
+#南京美食
+编辑于 4天前 江苏</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://sns-webpic-qc.xhscdn.com/202506132347/30b198824d4ed2fa2daa07a03cd6a543/notes_pre_post/1040g3k031igit4uhg8005pts32p3906ujbn2uco!nd_dft_wlteh_webp_3,https://sns-webpic-qc.xhscdn.com/202506132347/c9e9081173e9c7ba5754f1ecd12447f6/notes_pre_post/1040g3k031igit4uhg8005pts32p3906ujbn2uco!nd_prv_wlteh_webp_3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.xiaohongshu.com/search_result/68468cc8000000000c03a24e?xsec_token=AB9bh2lIaxSs4PxNygpmVS3sI4GlE2dcLhCsyWUd4tP-w=&amp;xsec_source=</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>